<commit_message>
consorcios subidos - no todos
</commit_message>
<xml_diff>
--- a/ALCORTA 146/Junio/JUNIO.xlsx
+++ b/ALCORTA 146/Junio/JUNIO.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Desktop\RC CONSORCIO 2025\ALCORTA 146\Junio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBF9FC68-341F-42DF-8F8B-20E8A87DF5A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{622578D9-9FEC-4C77-9FE1-62557460D557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="284" uniqueCount="203">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="202">
   <si>
     <t>LIQUIDACION DE EXPENSAS</t>
   </si>
@@ -591,24 +591,9 @@
     <t>FERNANDA</t>
   </si>
   <si>
-    <t>Salvatierra Matias -  Desobstruccion de cocina y baño en UF 3D</t>
-  </si>
-  <si>
-    <t>Cuota 5</t>
-  </si>
-  <si>
-    <t>Debito 07/05</t>
-  </si>
-  <si>
-    <t>Debito 12/05</t>
-  </si>
-  <si>
     <t>RUSSO</t>
   </si>
   <si>
-    <t>PREVISION ORDINARIA - ABONO VACACIONES ENCARGADO - ADEUDADAS</t>
-  </si>
-  <si>
     <t>VTO 14/07</t>
   </si>
   <si>
@@ -624,9 +609,6 @@
     <t xml:space="preserve">AYSA  - Mes de JUNIO </t>
   </si>
   <si>
-    <t>JUNIO</t>
-  </si>
-  <si>
     <t>Fumigacion -  JUNIO</t>
   </si>
   <si>
@@ -637,6 +619,21 @@
   </si>
   <si>
     <t>ARCA MES DE MAYO</t>
+  </si>
+  <si>
+    <t>EDESUR Nro de cliente : 01121995 - Mes de Mayo sin abonar</t>
+  </si>
+  <si>
+    <t>Cuota 6</t>
+  </si>
+  <si>
+    <t>Debito 12/06</t>
+  </si>
+  <si>
+    <t>Debito 09/06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PREVISION ORDINARIA </t>
   </si>
 </sst>
 </file>
@@ -1454,7 +1451,7 @@
     <xf numFmtId="166" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="189">
+  <cellXfs count="188">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -1624,6 +1621,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1666,11 +1666,35 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1686,30 +1710,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="20" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1734,10 +1734,6 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Millares" xfId="3" builtinId="3"/>
@@ -2168,7 +2164,7 @@
         <v>0</v>
       </c>
       <c r="B6" s="69" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="C6" s="69"/>
       <c r="D6" s="69" t="s">
@@ -2235,34 +2231,34 @@
       <c r="E14" s="71"/>
     </row>
     <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="146" t="s">
-        <v>193</v>
-      </c>
-      <c r="B15" s="146"/>
-      <c r="C15" s="146"/>
-      <c r="D15" s="146"/>
-      <c r="E15" s="146"/>
+      <c r="A15" s="147" t="s">
+        <v>188</v>
+      </c>
+      <c r="B15" s="147"/>
+      <c r="C15" s="147"/>
+      <c r="D15" s="147"/>
+      <c r="E15" s="147"/>
     </row>
     <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="146"/>
-      <c r="B16" s="146"/>
-      <c r="C16" s="146"/>
-      <c r="D16" s="146"/>
-      <c r="E16" s="146"/>
+      <c r="A16" s="147"/>
+      <c r="B16" s="147"/>
+      <c r="C16" s="147"/>
+      <c r="D16" s="147"/>
+      <c r="E16" s="147"/>
     </row>
     <row r="17" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="146"/>
-      <c r="B17" s="146"/>
-      <c r="C17" s="146"/>
-      <c r="D17" s="146"/>
-      <c r="E17" s="146"/>
+      <c r="A17" s="147"/>
+      <c r="B17" s="147"/>
+      <c r="C17" s="147"/>
+      <c r="D17" s="147"/>
+      <c r="E17" s="147"/>
     </row>
     <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="146"/>
-      <c r="B18" s="146"/>
-      <c r="C18" s="146"/>
-      <c r="D18" s="146"/>
-      <c r="E18" s="146"/>
+      <c r="A18" s="147"/>
+      <c r="B18" s="147"/>
+      <c r="C18" s="147"/>
+      <c r="D18" s="147"/>
+      <c r="E18" s="147"/>
     </row>
     <row r="19" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="71"/>
@@ -2286,39 +2282,39 @@
       <c r="E21" s="71"/>
     </row>
     <row r="22" spans="1:5" ht="0.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="147"/>
-      <c r="B22" s="148"/>
-      <c r="C22" s="148"/>
-      <c r="D22" s="148"/>
-      <c r="E22" s="148"/>
+      <c r="A22" s="148"/>
+      <c r="B22" s="149"/>
+      <c r="C22" s="149"/>
+      <c r="D22" s="149"/>
+      <c r="E22" s="149"/>
     </row>
     <row r="23" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="148"/>
-      <c r="B23" s="148"/>
-      <c r="C23" s="148"/>
-      <c r="D23" s="148"/>
-      <c r="E23" s="148"/>
+      <c r="A23" s="149"/>
+      <c r="B23" s="149"/>
+      <c r="C23" s="149"/>
+      <c r="D23" s="149"/>
+      <c r="E23" s="149"/>
     </row>
     <row r="24" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="148"/>
-      <c r="B24" s="148"/>
-      <c r="C24" s="148"/>
-      <c r="D24" s="148"/>
-      <c r="E24" s="148"/>
+      <c r="A24" s="149"/>
+      <c r="B24" s="149"/>
+      <c r="C24" s="149"/>
+      <c r="D24" s="149"/>
+      <c r="E24" s="149"/>
     </row>
     <row r="25" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="148"/>
-      <c r="B25" s="148"/>
-      <c r="C25" s="148"/>
-      <c r="D25" s="148"/>
-      <c r="E25" s="148"/>
+      <c r="A25" s="149"/>
+      <c r="B25" s="149"/>
+      <c r="C25" s="149"/>
+      <c r="D25" s="149"/>
+      <c r="E25" s="149"/>
     </row>
     <row r="26" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="148"/>
-      <c r="B26" s="148"/>
-      <c r="C26" s="148"/>
-      <c r="D26" s="148"/>
-      <c r="E26" s="148"/>
+      <c r="A26" s="149"/>
+      <c r="B26" s="149"/>
+      <c r="C26" s="149"/>
+      <c r="D26" s="149"/>
+      <c r="E26" s="149"/>
     </row>
     <row r="27" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="71"/>
@@ -2353,10 +2349,10 @@
         <v>127</v>
       </c>
       <c r="C30" s="78" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="D30" s="79">
-        <v>1664921.03</v>
+        <v>1612833.26</v>
       </c>
       <c r="E30" s="78"/>
     </row>
@@ -2367,7 +2363,7 @@
       </c>
       <c r="C31" s="78"/>
       <c r="D31" s="79">
-        <v>-362120.32</v>
+        <v>-350791.24</v>
       </c>
       <c r="E31" s="78"/>
     </row>
@@ -2378,7 +2374,7 @@
       </c>
       <c r="C32" s="78"/>
       <c r="D32" s="79">
-        <v>0.28999999999999998</v>
+        <v>0.98</v>
       </c>
       <c r="E32" s="78"/>
     </row>
@@ -2419,7 +2415,7 @@
       <c r="D37" s="82"/>
       <c r="E37" s="83">
         <f>SUM(D27:D34)</f>
-        <v>1302801</v>
+        <v>1262043</v>
       </c>
     </row>
     <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
@@ -2444,7 +2440,7 @@
       <c r="E39" s="78"/>
       <c r="G39" s="5">
         <f>E37+E41-G38</f>
-        <v>1067190</v>
+        <v>1026432</v>
       </c>
     </row>
     <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
@@ -2483,7 +2479,7 @@
         <v>142</v>
       </c>
       <c r="B43" s="78" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C43" s="78"/>
       <c r="D43" s="79">
@@ -2496,7 +2492,7 @@
         <v>143</v>
       </c>
       <c r="B44" s="78" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="C44" s="78"/>
       <c r="D44" s="79">
@@ -2541,7 +2537,7 @@
       </c>
       <c r="B48" s="78"/>
       <c r="C48" s="78" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="D48" s="17">
         <v>25842</v>
@@ -2578,28 +2574,28 @@
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" s="78" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B52" s="78"/>
       <c r="C52" s="78" t="s">
-        <v>189</v>
-      </c>
-      <c r="D52" s="187">
+        <v>200</v>
+      </c>
+      <c r="D52" s="17">
         <v>751741.52</v>
       </c>
       <c r="E52" s="24"/>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="78" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B53" s="78" t="s">
         <v>131</v>
       </c>
       <c r="C53" s="78" t="s">
-        <v>190</v>
-      </c>
-      <c r="D53" s="140">
+        <v>199</v>
+      </c>
+      <c r="D53" s="24">
         <v>72577.5</v>
       </c>
       <c r="E53" s="24"/>
@@ -2614,9 +2610,9 @@
       </c>
       <c r="C54" s="78" t="str">
         <f>C53</f>
-        <v>Debito 12/05</v>
-      </c>
-      <c r="D54" s="187">
+        <v>Debito 12/06</v>
+      </c>
+      <c r="D54" s="17">
         <v>128834.16</v>
       </c>
       <c r="E54" s="24"/>
@@ -2631,9 +2627,9 @@
       </c>
       <c r="C55" s="78" t="str">
         <f>C54</f>
-        <v>Debito 12/05</v>
-      </c>
-      <c r="D55" s="187">
+        <v>Debito 12/06</v>
+      </c>
+      <c r="D55" s="17">
         <v>8064.17</v>
       </c>
       <c r="E55" s="88"/>
@@ -2668,11 +2664,11 @@
     </row>
     <row r="59" spans="1:5" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="78" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="B59" s="92"/>
       <c r="C59" s="78"/>
-      <c r="D59" s="187">
+      <c r="D59" s="17">
         <v>472527.71</v>
       </c>
       <c r="E59" s="24"/>
@@ -2681,9 +2677,7 @@
       <c r="A60" s="92" t="s">
         <v>180</v>
       </c>
-      <c r="B60" s="92" t="s">
-        <v>198</v>
-      </c>
+      <c r="B60" s="92"/>
       <c r="C60" s="78"/>
       <c r="D60" s="17">
         <v>53800</v>
@@ -2703,12 +2697,12 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="78" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B62" s="78"/>
       <c r="C62" s="94"/>
       <c r="D62" s="17">
-        <v>45800</v>
+        <v>55000</v>
       </c>
       <c r="E62" s="24"/>
     </row>
@@ -2718,102 +2712,102 @@
       </c>
       <c r="B63" s="78"/>
       <c r="C63" s="78"/>
-      <c r="D63" s="187">
+      <c r="D63" s="17">
         <v>15389.22</v>
       </c>
       <c r="E63" s="24"/>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="78" t="s">
-        <v>119</v>
+        <v>197</v>
       </c>
       <c r="B64" s="78"/>
       <c r="C64" s="78"/>
-      <c r="D64" s="187">
-        <v>7181.14</v>
+      <c r="D64" s="17">
+        <v>189273.33</v>
       </c>
       <c r="E64" s="24"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="78" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="B65" s="78"/>
       <c r="C65" s="78"/>
-      <c r="D65" s="188">
-        <v>101821.18</v>
-      </c>
-      <c r="E65" s="143"/>
+      <c r="D65" s="17">
+        <v>7181.14</v>
+      </c>
+      <c r="E65" s="24"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" s="78" t="s">
-        <v>200</v>
+        <v>126</v>
       </c>
       <c r="B66" s="78"/>
       <c r="C66" s="78"/>
-      <c r="D66" s="187">
+      <c r="D66" s="145">
+        <v>101821.18</v>
+      </c>
+      <c r="E66" s="143"/>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="78" t="s">
+        <v>194</v>
+      </c>
+      <c r="B67" s="78"/>
+      <c r="C67" s="78"/>
+      <c r="D67" s="17">
         <v>16245.66</v>
       </c>
-      <c r="E66" s="24"/>
-    </row>
-    <row r="67" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="78"/>
-      <c r="B67" s="95"/>
-      <c r="C67" s="96"/>
-      <c r="D67" s="17"/>
-      <c r="E67" s="88"/>
+      <c r="E67" s="24"/>
     </row>
     <row r="68" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="20" t="s">
+      <c r="A68" s="78"/>
+      <c r="B68" s="95"/>
+      <c r="C68" s="96"/>
+      <c r="D68" s="17"/>
+      <c r="E68" s="88"/>
+    </row>
+    <row r="69" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A69" s="20" t="s">
         <v>5</v>
-      </c>
-      <c r="B68" s="20"/>
-      <c r="C68" s="20"/>
-      <c r="D68" s="25"/>
-      <c r="E68" s="89">
-        <f>SUM(D59:D67)</f>
-        <v>712764.91</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="19" t="s">
-        <v>116</v>
       </c>
       <c r="B69" s="20"/>
       <c r="C69" s="20"/>
       <c r="D69" s="25"/>
-      <c r="E69" s="89"/>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A70" s="78" t="s">
-        <v>162</v>
-      </c>
-      <c r="B70" s="78"/>
-      <c r="C70" s="78"/>
-      <c r="D70" s="17">
-        <v>44595</v>
-      </c>
-      <c r="E70" s="86"/>
+      <c r="E69" s="89">
+        <f>SUM(D59:D68)</f>
+        <v>911238.23999999987</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A70" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B70" s="20"/>
+      <c r="C70" s="20"/>
+      <c r="D70" s="25"/>
+      <c r="E70" s="89"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="78" t="s">
-        <v>181</v>
+        <v>162</v>
       </c>
       <c r="B71" s="78"/>
       <c r="C71" s="78"/>
       <c r="D71" s="17">
-        <v>52084.53</v>
-      </c>
-      <c r="E71" s="24"/>
+        <v>44595</v>
+      </c>
+      <c r="E71" s="86"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="78" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="B72" s="78"/>
       <c r="C72" s="78"/>
       <c r="D72" s="17">
-        <v>45800</v>
+        <v>52084.53</v>
       </c>
       <c r="E72" s="24"/>
     </row>
@@ -2843,8 +2837,8 @@
       <c r="C75" s="19"/>
       <c r="D75" s="19"/>
       <c r="E75" s="97">
-        <f>SUM(D70:D74)</f>
-        <v>144829.53</v>
+        <f>SUM(D71:D74)</f>
+        <v>99029.53</v>
       </c>
     </row>
     <row r="76" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2863,8 +2857,8 @@
       <c r="B77" s="78"/>
       <c r="C77" s="78"/>
       <c r="D77" s="17">
-        <f>52561.98+29000</f>
-        <v>81561.98000000001</v>
+        <f>55821.88+14500</f>
+        <v>70321.88</v>
       </c>
       <c r="E77" s="98"/>
     </row>
@@ -2884,7 +2878,7 @@
       <c r="D79" s="12"/>
       <c r="E79" s="89">
         <f>SUM(D77:D78)</f>
-        <v>81561.98000000001</v>
+        <v>70321.88</v>
       </c>
     </row>
     <row r="80" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2896,13 +2890,13 @@
     </row>
     <row r="81" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A81" s="101" t="s">
-        <v>192</v>
+        <v>201</v>
       </c>
       <c r="B81" s="101"/>
       <c r="C81" s="101"/>
       <c r="D81" s="102"/>
       <c r="E81" s="103">
-        <v>1700000</v>
+        <v>4000000</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2922,7 +2916,7 @@
       <c r="D83" s="108"/>
       <c r="E83" s="109">
         <f>(SUM(E30:E81))</f>
-        <v>5069016.7699999996</v>
+        <v>7469692</v>
       </c>
       <c r="F83" s="31"/>
       <c r="G83" s="31"/>
@@ -2943,40 +2937,40 @@
       <c r="F85" s="31"/>
     </row>
     <row r="86" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A86" s="157" t="s">
+      <c r="A86" s="158" t="s">
         <v>158</v>
       </c>
-      <c r="B86" s="158"/>
+      <c r="B86" s="159"/>
       <c r="C86" s="110"/>
       <c r="D86" s="71"/>
       <c r="E86" s="71"/>
     </row>
     <row r="87" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="149"/>
-      <c r="B87" s="150"/>
+      <c r="A87" s="150"/>
+      <c r="B87" s="151"/>
       <c r="C87" s="17"/>
       <c r="D87" s="71"/>
       <c r="E87" s="71"/>
     </row>
     <row r="88" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A88" s="151"/>
-      <c r="B88" s="152"/>
+      <c r="A88" s="152"/>
+      <c r="B88" s="153"/>
       <c r="C88" s="17"/>
       <c r="D88" s="71"/>
       <c r="E88" s="71"/>
     </row>
     <row r="89" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A89" s="153"/>
-      <c r="B89" s="154"/>
+      <c r="A89" s="154"/>
+      <c r="B89" s="155"/>
       <c r="C89" s="111"/>
       <c r="D89" s="71"/>
       <c r="E89" s="112"/>
     </row>
     <row r="90" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="155" t="s">
+      <c r="A90" s="156" t="s">
         <v>16</v>
       </c>
-      <c r="B90" s="156"/>
+      <c r="B90" s="157"/>
       <c r="C90" s="113">
         <f>SUM(C87:C89)</f>
         <v>0</v>
@@ -3013,7 +3007,7 @@
       </c>
       <c r="B94" s="118">
         <f>E83</f>
-        <v>5069016.7699999996</v>
+        <v>7469692</v>
       </c>
       <c r="C94" s="71"/>
       <c r="D94" s="71"/>
@@ -3025,7 +3019,7 @@
       </c>
       <c r="B95" s="120">
         <f>E83-E81</f>
-        <v>3369016.7699999996</v>
+        <v>3469692</v>
       </c>
       <c r="C95" s="71"/>
       <c r="D95" s="71"/>
@@ -3061,7 +3055,7 @@
       </c>
       <c r="B98" s="122">
         <f>B95+B97</f>
-        <v>3369016.7699999996</v>
+        <v>3469692</v>
       </c>
       <c r="C98" s="71"/>
       <c r="D98" s="71"/>
@@ -3075,16 +3069,16 @@
       <c r="E99" s="71"/>
     </row>
     <row r="100" spans="1:5" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A100" s="148"/>
-      <c r="B100" s="148"/>
-      <c r="C100" s="148"/>
+      <c r="A100" s="149"/>
+      <c r="B100" s="149"/>
+      <c r="C100" s="149"/>
       <c r="D100" s="71"/>
       <c r="E100" s="71"/>
     </row>
     <row r="101" spans="1:5" ht="35.25" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A101" s="148"/>
-      <c r="B101" s="148"/>
-      <c r="C101" s="148"/>
+      <c r="A101" s="149"/>
+      <c r="B101" s="149"/>
+      <c r="C101" s="149"/>
       <c r="D101" s="71"/>
       <c r="E101" s="71"/>
     </row>
@@ -3109,7 +3103,7 @@
         <v>42</v>
       </c>
       <c r="B104" s="124">
-        <v>-28063.224127181806</v>
+        <v>242274.94714675145</v>
       </c>
       <c r="C104" s="126"/>
       <c r="D104" s="71"/>
@@ -3121,7 +3115,7 @@
       </c>
       <c r="B105" s="128">
         <f>PRORRATEO!I44</f>
-        <v>2822724.5812739334</v>
+        <v>3413182.0317890993</v>
       </c>
       <c r="C105" s="125"/>
       <c r="D105" s="112"/>
@@ -3133,7 +3127,7 @@
       </c>
       <c r="B106" s="142">
         <f>-(B98+B114)</f>
-        <v>-3019055.7699999996</v>
+        <v>-3119731</v>
       </c>
       <c r="C106" s="125"/>
       <c r="D106" s="71"/>
@@ -3145,7 +3139,7 @@
       </c>
       <c r="B107" s="42">
         <f>SUM(B104:B106)</f>
-        <v>-224394.41285324795</v>
+        <v>535725.97893585078</v>
       </c>
       <c r="C107" s="131"/>
       <c r="D107" s="112"/>
@@ -3186,7 +3180,7 @@
         <v>42</v>
       </c>
       <c r="B112" s="24">
-        <v>331375.87932759989</v>
+        <v>436123.85052585986</v>
       </c>
       <c r="C112" s="134"/>
       <c r="D112" s="137"/>
@@ -3198,7 +3192,7 @@
       </c>
       <c r="B113" s="24">
         <f>PRORRATEO!I45</f>
-        <v>454708.97119825997</v>
+        <v>528808.55360800005</v>
       </c>
       <c r="C113" s="131"/>
       <c r="D113" s="112"/>
@@ -3243,7 +3237,7 @@
       </c>
       <c r="B118" s="42">
         <f>SUM(B112:B117)</f>
-        <v>436123.85052585986</v>
+        <v>614971.40413385991</v>
       </c>
       <c r="C118" s="125"/>
       <c r="D118" s="71"/>
@@ -3257,16 +3251,16 @@
       <c r="E119" s="71"/>
     </row>
     <row r="121" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A121" s="145" t="s">
+      <c r="A121" s="146" t="s">
         <v>164</v>
       </c>
-      <c r="B121" s="145"/>
-      <c r="C121" s="145"/>
+      <c r="B121" s="146"/>
+      <c r="C121" s="146"/>
     </row>
     <row r="122" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A122" s="145"/>
-      <c r="B122" s="145"/>
-      <c r="C122" s="145"/>
+      <c r="A122" s="146"/>
+      <c r="B122" s="146"/>
+      <c r="C122" s="146"/>
     </row>
     <row r="123" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A123" s="1"/>
@@ -3324,7 +3318,7 @@
     <col min="13" max="13" width="5" hidden="1" customWidth="1"/>
     <col min="14" max="14" width="14.7109375" customWidth="1"/>
     <col min="15" max="15" width="14.5703125" customWidth="1"/>
-    <col min="17" max="17" width="12" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -3364,7 +3358,7 @@
         <v>2902347.4099999997</v>
       </c>
       <c r="O2" s="39">
-        <v>4602347.41</v>
+        <v>7469692</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
@@ -3383,11 +3377,11 @@
       </c>
       <c r="L3" s="2"/>
       <c r="M3" s="2"/>
-      <c r="N3" s="168">
+      <c r="N3" s="162">
         <f>O2</f>
-        <v>4602347.41</v>
-      </c>
-      <c r="O3" s="168"/>
+        <v>7469692</v>
+      </c>
+      <c r="O3" s="162"/>
       <c r="P3" s="5"/>
     </row>
     <row r="4" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3406,70 +3400,70 @@
       </c>
       <c r="L4" s="2"/>
       <c r="M4" s="2"/>
-      <c r="N4" s="167"/>
-      <c r="O4" s="167"/>
+      <c r="N4" s="161"/>
+      <c r="O4" s="161"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" s="159" t="s">
+      <c r="A5" s="163" t="s">
         <v>8</v>
       </c>
-      <c r="B5" s="161" t="s">
+      <c r="B5" s="170" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="163" t="s">
+      <c r="C5" s="172" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="163" t="s">
+      <c r="D5" s="172" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="163" t="s">
+      <c r="E5" s="172" t="s">
         <v>132</v>
       </c>
-      <c r="F5" s="159" t="s">
+      <c r="F5" s="163" t="s">
         <v>37</v>
       </c>
-      <c r="G5" s="159" t="s">
+      <c r="G5" s="163" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="159" t="s">
+      <c r="H5" s="163" t="s">
         <v>13</v>
       </c>
       <c r="I5" s="14"/>
-      <c r="J5" s="171" t="s">
+      <c r="J5" s="167" t="s">
         <v>147</v>
       </c>
-      <c r="K5" s="169" t="s">
+      <c r="K5" s="165" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="169" t="s">
+      <c r="L5" s="165" t="s">
         <v>33</v>
       </c>
-      <c r="M5" s="169" t="s">
+      <c r="M5" s="165" t="s">
         <v>15</v>
       </c>
-      <c r="N5" s="169" t="s">
+      <c r="N5" s="165" t="s">
         <v>31</v>
       </c>
-      <c r="O5" s="169" t="s">
+      <c r="O5" s="165" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A6" s="160"/>
-      <c r="B6" s="162"/>
-      <c r="C6" s="164"/>
-      <c r="D6" s="164"/>
-      <c r="E6" s="165"/>
-      <c r="F6" s="160"/>
-      <c r="G6" s="160"/>
-      <c r="H6" s="160"/>
+      <c r="A6" s="164"/>
+      <c r="B6" s="171"/>
+      <c r="C6" s="173"/>
+      <c r="D6" s="173"/>
+      <c r="E6" s="174"/>
+      <c r="F6" s="164"/>
+      <c r="G6" s="164"/>
+      <c r="H6" s="164"/>
       <c r="I6" s="15"/>
-      <c r="J6" s="172"/>
-      <c r="K6" s="170"/>
-      <c r="L6" s="173"/>
-      <c r="M6" s="173"/>
-      <c r="N6" s="173"/>
-      <c r="O6" s="170"/>
+      <c r="J6" s="168"/>
+      <c r="K6" s="166"/>
+      <c r="L6" s="169"/>
+      <c r="M6" s="169"/>
+      <c r="N6" s="169"/>
+      <c r="O6" s="166"/>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -3487,18 +3481,18 @@
         <v>2.63</v>
       </c>
       <c r="G7" s="24">
-        <v>104080.23140012554</v>
+        <v>121040.87763392553</v>
       </c>
       <c r="H7" s="29">
-        <f>168983-G39</f>
-        <v>104081.09064920002</v>
+        <f>168983+27536-G39</f>
+        <v>121040.50247600001</v>
       </c>
       <c r="I7" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J7" s="7">
         <f>H7-G7</f>
-        <v>0.85924907447770238</v>
+        <v>-0.37515792551857885</v>
       </c>
       <c r="K7" s="40">
         <f>N$4*F7%</f>
@@ -3506,16 +3500,16 @@
       </c>
       <c r="L7" s="6">
         <f>N$3*F7%</f>
-        <v>121041.73688300001</v>
+        <v>196452.8996</v>
       </c>
       <c r="M7" s="23"/>
       <c r="N7" s="23">
         <f>L7+K7-J7+M7</f>
-        <v>121040.87763392553</v>
+        <v>196453.27475792554</v>
       </c>
       <c r="O7" s="23">
         <f>N7*6% + N7</f>
-        <v>128303.33029196106</v>
+        <v>208240.47124340106</v>
       </c>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
@@ -3536,18 +3530,18 @@
         <v>3.33</v>
       </c>
       <c r="G8" s="24">
-        <v>349862.72621394927</v>
+        <v>371337.89496694924</v>
       </c>
       <c r="H8" s="29">
-        <f>131783</f>
-        <v>131783</v>
+        <f>153258</f>
+        <v>153258</v>
       </c>
       <c r="I8" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J8" s="7">
         <f t="shared" ref="J8:J42" si="0">H8-G8</f>
-        <v>-218079.72621394927</v>
+        <v>-218079.89496694924</v>
       </c>
       <c r="K8" s="40">
         <f t="shared" ref="K8:K42" si="1">N$4*F8%</f>
@@ -3555,18 +3549,21 @@
       </c>
       <c r="L8" s="6">
         <f t="shared" ref="L8:L42" si="2">N$3*F8%</f>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M8" s="23"/>
       <c r="N8" s="23">
         <f>L8+K8-J8+M8</f>
-        <v>371337.89496694924</v>
+        <v>466820.63856694929</v>
       </c>
       <c r="O8" s="23">
         <f t="shared" ref="O8:O42" si="3">N8*6% + N8</f>
-        <v>393618.16866496619</v>
-      </c>
-      <c r="Q8" s="31"/>
+        <v>494829.87688096624</v>
+      </c>
+      <c r="Q8" s="31">
+        <f>G7+G39</f>
+        <v>196519.37515792553</v>
+      </c>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -3584,18 +3581,18 @@
         <v>3.32</v>
       </c>
       <c r="G9" s="24">
-        <v>131387.14420079993</v>
+        <v>152797.63821279994</v>
       </c>
       <c r="H9" s="29">
-        <f>99904.44+31482+1</f>
-        <v>131387.44</v>
+        <f>G9</f>
+        <v>152797.63821279994</v>
       </c>
       <c r="I9" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J9" s="7">
         <f t="shared" si="0"/>
-        <v>0.29579920007381588</v>
+        <v>0</v>
       </c>
       <c r="K9" s="40">
         <f t="shared" si="1"/>
@@ -3603,16 +3600,16 @@
       </c>
       <c r="L9" s="6">
         <f t="shared" si="2"/>
-        <v>152797.93401200001</v>
+        <v>247993.77439999999</v>
       </c>
       <c r="M9" s="23"/>
       <c r="N9" s="23">
         <f t="shared" ref="N9:N42" si="4">L9+K9-J9+M9</f>
-        <v>152797.63821279994</v>
+        <v>247993.77439999999</v>
       </c>
       <c r="O9" s="23">
         <f t="shared" si="3"/>
-        <v>161965.49650556792</v>
+        <v>262873.40086399997</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.25">
@@ -3631,18 +3628,18 @@
         <v>3.42</v>
       </c>
       <c r="G10" s="24">
-        <v>490761.9139134034</v>
+        <v>512162.19533540343</v>
       </c>
       <c r="H10" s="29">
-        <f>136000</f>
-        <v>136000</v>
+        <f>150000+7500</f>
+        <v>157500</v>
       </c>
       <c r="I10" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J10" s="7">
         <f t="shared" si="0"/>
-        <v>-354761.9139134034</v>
+        <v>-354662.19533540343</v>
       </c>
       <c r="K10" s="40">
         <f t="shared" si="1"/>
@@ -3650,16 +3647,16 @@
       </c>
       <c r="L10" s="6">
         <f t="shared" si="2"/>
-        <v>157400.281422</v>
+        <v>255463.4664</v>
       </c>
       <c r="M10" s="23"/>
       <c r="N10" s="23">
         <f t="shared" si="4"/>
-        <v>512162.19533540343</v>
+        <v>610125.66173540347</v>
       </c>
       <c r="O10" s="23">
         <f t="shared" si="3"/>
-        <v>542891.92705552769</v>
+        <v>646733.20143952768</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.25">
@@ -3678,11 +3675,11 @@
         <v>3.34</v>
       </c>
       <c r="G11" s="24">
-        <v>132178.27879979997</v>
+        <v>153718.403494</v>
       </c>
       <c r="H11" s="29">
         <f>G11</f>
-        <v>132178.27879979997</v>
+        <v>153718.403494</v>
       </c>
       <c r="I11" s="13" t="s">
         <v>123</v>
@@ -3697,16 +3694,16 @@
       </c>
       <c r="L11" s="6">
         <f t="shared" si="2"/>
-        <v>153718.403494</v>
+        <v>249487.71279999998</v>
       </c>
       <c r="M11" s="23"/>
       <c r="N11" s="23">
         <f t="shared" si="4"/>
-        <v>153718.403494</v>
+        <v>249487.71279999998</v>
       </c>
       <c r="O11" s="23">
         <f t="shared" si="3"/>
-        <v>162941.50770364</v>
+        <v>264456.97556799999</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.25">
@@ -3725,11 +3722,11 @@
         <v>3.33</v>
       </c>
       <c r="G12" s="24">
-        <v>131782.53545009997</v>
+        <v>153258.16875300001</v>
       </c>
       <c r="H12" s="29">
         <f>G12</f>
-        <v>131782.53545009997</v>
+        <v>153258.16875300001</v>
       </c>
       <c r="I12" s="13" t="s">
         <v>123</v>
@@ -3744,16 +3741,16 @@
       </c>
       <c r="L12" s="6">
         <f t="shared" si="2"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M12" s="23"/>
       <c r="N12" s="23">
         <f t="shared" si="4"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="O12" s="23">
         <f t="shared" si="3"/>
-        <v>162453.65887817999</v>
+        <v>263665.18821600004</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.25">
@@ -3772,11 +3769,11 @@
         <v>3.32</v>
       </c>
       <c r="G13" s="24">
-        <v>131386.79210039997</v>
+        <v>152797.93401200001</v>
       </c>
       <c r="H13" s="29">
         <f>G13</f>
-        <v>131386.79210039997</v>
+        <v>152797.93401200001</v>
       </c>
       <c r="I13" s="13" t="s">
         <v>123</v>
@@ -3791,16 +3788,16 @@
       </c>
       <c r="L13" s="6">
         <f t="shared" si="2"/>
-        <v>152797.93401200001</v>
+        <v>247993.77439999999</v>
       </c>
       <c r="M13" s="23"/>
       <c r="N13" s="23">
         <f t="shared" si="4"/>
-        <v>152797.93401200001</v>
+        <v>247993.77439999999</v>
       </c>
       <c r="O13" s="23">
         <f t="shared" si="3"/>
-        <v>161965.81005272001</v>
+        <v>262873.40086399997</v>
       </c>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.25">
@@ -3819,11 +3816,11 @@
         <v>3.33</v>
       </c>
       <c r="G14" s="24">
-        <v>131782.53090019993</v>
+        <v>153258.16875300001</v>
       </c>
       <c r="H14" s="29">
         <f>G14</f>
-        <v>131782.53090019993</v>
+        <v>153258.16875300001</v>
       </c>
       <c r="I14" s="13" t="s">
         <v>123</v>
@@ -3838,16 +3835,16 @@
       </c>
       <c r="L14" s="6">
         <f t="shared" si="2"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M14" s="23"/>
       <c r="N14" s="23">
         <f t="shared" si="4"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="O14" s="23">
         <f t="shared" si="3"/>
-        <v>162453.65887817999</v>
+        <v>263665.18821600004</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.25">
@@ -3868,7 +3865,7 @@
         <v>3.24</v>
       </c>
       <c r="G15" s="24">
-        <v>204755.73604600481</v>
+        <v>225650.79213000485</v>
       </c>
       <c r="H15" s="29">
         <v>128221</v>
@@ -3878,7 +3875,7 @@
       </c>
       <c r="J15" s="7">
         <f t="shared" si="0"/>
-        <v>-76534.736046004808</v>
+        <v>-97429.792130004847</v>
       </c>
       <c r="K15" s="40">
         <f t="shared" si="1"/>
@@ -3886,16 +3883,16 @@
       </c>
       <c r="L15" s="6">
         <f t="shared" si="2"/>
-        <v>149116.05608400004</v>
+        <v>242018.02080000003</v>
       </c>
       <c r="M15" s="23"/>
       <c r="N15" s="23">
         <f t="shared" si="4"/>
-        <v>225650.79213000485</v>
+        <v>339447.8129300049</v>
       </c>
       <c r="O15" s="23">
         <f t="shared" si="3"/>
-        <v>239189.83965780513</v>
+        <v>359814.68170580518</v>
       </c>
       <c r="R15" t="s">
         <v>184</v>
@@ -3919,7 +3916,7 @@
         <v>3.33</v>
       </c>
       <c r="G16" s="24">
-        <v>263565.07090019993</v>
+        <v>416823.23965319991</v>
       </c>
       <c r="H16" s="29"/>
       <c r="I16" s="13" t="s">
@@ -3927,7 +3924,7 @@
       </c>
       <c r="J16" s="7">
         <f t="shared" si="0"/>
-        <v>-263565.07090019993</v>
+        <v>-416823.23965319991</v>
       </c>
       <c r="K16" s="40">
         <f t="shared" si="1"/>
@@ -3935,16 +3932,16 @@
       </c>
       <c r="L16" s="6">
         <f t="shared" si="2"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M16" s="23"/>
       <c r="N16" s="23">
         <f>L16+K16-J16+M16</f>
-        <v>416823.23965319991</v>
+        <v>665563.98325319996</v>
       </c>
       <c r="O16" s="23">
         <f t="shared" si="3"/>
-        <v>441832.63403239188</v>
+        <v>705497.82224839192</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.25">
@@ -3963,18 +3960,17 @@
         <v>3.32</v>
       </c>
       <c r="G17" s="24">
-        <v>131386.79210039997</v>
+        <v>161965.81005272001</v>
       </c>
       <c r="H17" s="29">
-        <f>G17</f>
-        <v>131386.79210039997</v>
+        <v>152797.23000000001</v>
       </c>
       <c r="I17" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J17" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-9168.5800527200045</v>
       </c>
       <c r="K17" s="40">
         <f t="shared" si="1"/>
@@ -3982,16 +3978,16 @@
       </c>
       <c r="L17" s="6">
         <f t="shared" si="2"/>
-        <v>152797.93401200001</v>
+        <v>247993.77439999999</v>
       </c>
       <c r="M17" s="23"/>
       <c r="N17" s="23">
         <f t="shared" si="4"/>
-        <v>152797.93401200001</v>
+        <v>257162.35445272</v>
       </c>
       <c r="O17" s="23">
         <f t="shared" si="3"/>
-        <v>161965.81005272001</v>
+        <v>272592.09571988322</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.25">
@@ -4010,18 +4006,18 @@
         <v>3.33</v>
       </c>
       <c r="G18" s="24">
-        <v>241782.07481739999</v>
+        <v>365040.24357039999</v>
       </c>
       <c r="H18" s="29">
-        <f>30000</f>
-        <v>30000</v>
+        <f>50040.24+316000</f>
+        <v>366040.24</v>
       </c>
       <c r="I18" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J18" s="7">
         <f t="shared" si="0"/>
-        <v>-211782.07481739999</v>
+        <v>999.99642959999619</v>
       </c>
       <c r="K18" s="40">
         <f t="shared" si="1"/>
@@ -4029,16 +4025,16 @@
       </c>
       <c r="L18" s="6">
         <f t="shared" si="2"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M18" s="23"/>
       <c r="N18" s="23">
         <f t="shared" si="4"/>
-        <v>365040.24357039999</v>
+        <v>247740.74717040002</v>
       </c>
       <c r="O18" s="23">
         <f t="shared" si="3"/>
-        <v>386942.65818462399</v>
+        <v>262605.19200062403</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.25">
@@ -4057,18 +4053,18 @@
         <v>3.24</v>
       </c>
       <c r="G19" s="24">
-        <v>128196.94419997238</v>
+        <v>149214.9096347724</v>
       </c>
       <c r="H19" s="29">
-        <f>193000-H32</f>
-        <v>128098.09064920002</v>
+        <f>224700-H32</f>
+        <v>149221.50247599999</v>
       </c>
       <c r="I19" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J19" s="7">
         <f t="shared" si="0"/>
-        <v>-98.853550772357266</v>
+        <v>6.5928412275970913</v>
       </c>
       <c r="K19" s="40">
         <f t="shared" si="1"/>
@@ -4076,16 +4072,16 @@
       </c>
       <c r="L19" s="6">
         <f t="shared" si="2"/>
-        <v>149116.05608400004</v>
+        <v>242018.02080000003</v>
       </c>
       <c r="M19" s="23"/>
       <c r="N19" s="23">
         <f t="shared" si="4"/>
-        <v>149214.9096347724</v>
+        <v>242011.42795877243</v>
       </c>
       <c r="O19" s="23">
         <f t="shared" si="3"/>
-        <v>158167.80421285873</v>
+        <v>256532.11363629877</v>
       </c>
     </row>
     <row r="20" spans="1:18" x14ac:dyDescent="0.25">
@@ -4106,17 +4102,18 @@
         <v>3.33</v>
       </c>
       <c r="G20" s="24">
-        <v>139799.86545009995</v>
+        <v>153058.03420309996</v>
       </c>
       <c r="H20" s="29">
-        <v>140000</v>
+        <f>G20</f>
+        <v>153058.03420309996</v>
       </c>
       <c r="I20" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J20" s="7">
         <f t="shared" si="0"/>
-        <v>200.13454990004539</v>
+        <v>0</v>
       </c>
       <c r="K20" s="40">
         <f t="shared" si="1"/>
@@ -4124,16 +4121,16 @@
       </c>
       <c r="L20" s="6">
         <f t="shared" si="2"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M20" s="23"/>
       <c r="N20" s="23">
         <f t="shared" si="4"/>
-        <v>153058.03420309996</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="O20" s="23">
         <f t="shared" si="3"/>
-        <v>162241.51625528597</v>
+        <v>263665.18821600004</v>
       </c>
     </row>
     <row r="21" spans="1:18" x14ac:dyDescent="0.25">
@@ -4152,7 +4149,7 @@
         <v>3.32</v>
       </c>
       <c r="G21" s="24">
-        <v>323774.00456925598</v>
+        <v>476571.93858125596</v>
       </c>
       <c r="H21" s="29"/>
       <c r="I21" s="13" t="s">
@@ -4160,7 +4157,7 @@
       </c>
       <c r="J21" s="7">
         <f>H21-G21</f>
-        <v>-323774.00456925598</v>
+        <v>-476571.93858125596</v>
       </c>
       <c r="K21" s="40">
         <f t="shared" si="1"/>
@@ -4168,16 +4165,16 @@
       </c>
       <c r="L21" s="6">
         <f t="shared" si="2"/>
-        <v>152797.93401200001</v>
+        <v>247993.77439999999</v>
       </c>
       <c r="M21" s="23"/>
       <c r="N21" s="23">
         <f t="shared" si="4"/>
-        <v>476571.93858125596</v>
+        <v>724565.71298125596</v>
       </c>
       <c r="O21" s="23">
         <f t="shared" si="3"/>
-        <v>505166.25489613134</v>
+        <v>768039.65576013131</v>
       </c>
     </row>
     <row r="22" spans="1:18" x14ac:dyDescent="0.25">
@@ -4196,7 +4193,7 @@
         <v>3.33</v>
       </c>
       <c r="G22" s="13">
-        <v>1863887.0562139489</v>
+        <v>2017145.2249669489</v>
       </c>
       <c r="H22" s="29"/>
       <c r="I22" s="13" t="s">
@@ -4204,7 +4201,7 @@
       </c>
       <c r="J22" s="43">
         <f t="shared" si="0"/>
-        <v>-1863887.0562139489</v>
+        <v>-2017145.2249669489</v>
       </c>
       <c r="K22" s="40">
         <f t="shared" si="1"/>
@@ -4212,16 +4209,16 @@
       </c>
       <c r="L22" s="6">
         <f t="shared" si="2"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M22" s="23"/>
       <c r="N22" s="23">
         <f t="shared" si="4"/>
-        <v>2017145.2249669489</v>
+        <v>2265885.968566949</v>
       </c>
       <c r="O22" s="23">
         <f t="shared" si="3"/>
-        <v>2138173.9384649657</v>
+        <v>2401839.126680966</v>
       </c>
       <c r="R22" s="30"/>
     </row>
@@ -4243,11 +4240,11 @@
         <v>3.24</v>
       </c>
       <c r="G23" s="24">
-        <v>128220.70769576005</v>
+        <v>149116.05608400004</v>
       </c>
       <c r="H23" s="29">
         <f>G23</f>
-        <v>128220.70769576005</v>
+        <v>149116.05608400004</v>
       </c>
       <c r="I23" s="13" t="s">
         <v>140</v>
@@ -4262,16 +4259,16 @@
       </c>
       <c r="L23" s="6">
         <f t="shared" si="2"/>
-        <v>149116.05608400004</v>
+        <v>242018.02080000003</v>
       </c>
       <c r="M23" s="23"/>
       <c r="N23" s="23">
         <f t="shared" si="4"/>
-        <v>149116.05608400004</v>
+        <v>242018.02080000003</v>
       </c>
       <c r="O23" s="23">
         <f t="shared" si="3"/>
-        <v>158063.01944904003</v>
+        <v>256539.10204800003</v>
       </c>
     </row>
     <row r="24" spans="1:18" x14ac:dyDescent="0.25">
@@ -4290,17 +4287,18 @@
         <v>3.24</v>
       </c>
       <c r="G24" s="24">
-        <v>121017.76468720005</v>
+        <v>141133.82077120009</v>
       </c>
       <c r="H24" s="29">
-        <v>129000</v>
+        <f>G24</f>
+        <v>141133.82077120009</v>
       </c>
       <c r="I24" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J24" s="7">
         <f t="shared" si="0"/>
-        <v>7982.2353127999522</v>
+        <v>0</v>
       </c>
       <c r="K24" s="40">
         <f t="shared" si="1"/>
@@ -4308,16 +4306,16 @@
       </c>
       <c r="L24" s="6">
         <f t="shared" si="2"/>
-        <v>149116.05608400004</v>
+        <v>242018.02080000003</v>
       </c>
       <c r="M24" s="23"/>
       <c r="N24" s="23">
         <f t="shared" si="4"/>
-        <v>141133.82077120009</v>
+        <v>242018.02080000003</v>
       </c>
       <c r="O24" s="23">
         <f t="shared" si="3"/>
-        <v>149601.85001747208</v>
+        <v>256539.10204800003</v>
       </c>
     </row>
     <row r="25" spans="1:18" x14ac:dyDescent="0.25">
@@ -4338,18 +4336,18 @@
         <v>3.32</v>
       </c>
       <c r="G25" s="24">
-        <v>131388.69066119989</v>
+        <v>152798.53402399988</v>
       </c>
       <c r="H25" s="29">
-        <f>196290-H33</f>
-        <v>131388.09064920002</v>
+        <f>228278-H33</f>
+        <v>152799.50247599999</v>
       </c>
       <c r="I25" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J25" s="7">
         <f t="shared" si="0"/>
-        <v>-0.60001199986436404</v>
+        <v>0.96845200011739507</v>
       </c>
       <c r="K25" s="40">
         <f t="shared" si="1"/>
@@ -4357,16 +4355,16 @@
       </c>
       <c r="L25" s="6">
         <f t="shared" si="2"/>
-        <v>152797.93401200001</v>
+        <v>247993.77439999999</v>
       </c>
       <c r="M25" s="23"/>
       <c r="N25" s="23">
         <f t="shared" si="4"/>
-        <v>152798.53402399988</v>
+        <v>247992.80594799988</v>
       </c>
       <c r="O25" s="23">
         <f t="shared" si="3"/>
-        <v>161966.44606543987</v>
+        <v>262872.37430487986</v>
       </c>
     </row>
     <row r="26" spans="1:18" x14ac:dyDescent="0.25">
@@ -4387,11 +4385,11 @@
         <v>3.33</v>
       </c>
       <c r="G26" s="17">
-        <v>131782.53545009997</v>
+        <v>153258.16875300001</v>
       </c>
       <c r="H26" s="29">
         <f>G26</f>
-        <v>131782.53545009997</v>
+        <v>153258.16875300001</v>
       </c>
       <c r="I26" s="13" t="s">
         <v>123</v>
@@ -4406,16 +4404,16 @@
       </c>
       <c r="L26" s="6">
         <f t="shared" si="2"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M26" s="23"/>
       <c r="N26" s="23">
         <f t="shared" si="4"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="O26" s="23">
         <f t="shared" si="3"/>
-        <v>162453.65887817999</v>
+        <v>263665.18821600004</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.25">
@@ -4436,11 +4434,11 @@
         <v>3.24</v>
       </c>
       <c r="G27" s="24">
-        <v>128221.14102283421</v>
+        <v>149116.05608400004</v>
       </c>
       <c r="H27" s="29">
         <f>G27</f>
-        <v>128221.14102283421</v>
+        <v>149116.05608400004</v>
       </c>
       <c r="I27" s="13" t="s">
         <v>152</v>
@@ -4455,16 +4453,16 @@
       </c>
       <c r="L27" s="6">
         <f t="shared" si="2"/>
-        <v>149116.05608400004</v>
+        <v>242018.02080000003</v>
       </c>
       <c r="M27" s="23"/>
       <c r="N27" s="23">
         <f t="shared" si="4"/>
-        <v>149116.05608400004</v>
+        <v>242018.02080000003</v>
       </c>
       <c r="O27" s="23">
         <f t="shared" si="3"/>
-        <v>158063.01944904003</v>
+        <v>256539.10204800003</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.25">
@@ -4483,18 +4481,18 @@
         <v>3.33</v>
       </c>
       <c r="G28" s="24">
-        <v>131782.53545009997</v>
+        <v>153258.16875300001</v>
       </c>
       <c r="H28" s="29">
-        <f>G28</f>
-        <v>131782.53545009997</v>
+        <f>304214-H37-H36</f>
+        <v>153257.00495199999</v>
       </c>
       <c r="I28" s="13" t="s">
         <v>124</v>
       </c>
       <c r="J28" s="7">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>-1.1638010000169743</v>
       </c>
       <c r="K28" s="40">
         <f t="shared" si="1"/>
@@ -4502,16 +4500,16 @@
       </c>
       <c r="L28" s="6">
         <f t="shared" si="2"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M28" s="23"/>
       <c r="N28" s="23">
         <f t="shared" si="4"/>
-        <v>153258.16875300001</v>
+        <v>248741.90740100003</v>
       </c>
       <c r="O28" s="23">
         <f t="shared" si="3"/>
-        <v>162453.65887817999</v>
+        <v>263666.42184506002</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.25">
@@ -4530,7 +4528,7 @@
         <v>3.32</v>
       </c>
       <c r="G29" s="24">
-        <v>131386.79210039997</v>
+        <v>284184.72611239995</v>
       </c>
       <c r="H29" s="29"/>
       <c r="I29" s="13" t="s">
@@ -4538,7 +4536,7 @@
       </c>
       <c r="J29" s="7">
         <f t="shared" si="0"/>
-        <v>-131386.79210039997</v>
+        <v>-284184.72611239995</v>
       </c>
       <c r="K29" s="40">
         <f t="shared" si="1"/>
@@ -4546,16 +4544,16 @@
       </c>
       <c r="L29" s="6">
         <f t="shared" si="2"/>
-        <v>152797.93401200001</v>
+        <v>247993.77439999999</v>
       </c>
       <c r="M29" s="23"/>
       <c r="N29" s="23">
         <f t="shared" si="4"/>
-        <v>284184.72611239995</v>
+        <v>532178.50051239994</v>
       </c>
       <c r="O29" s="23">
         <f t="shared" si="3"/>
-        <v>301235.80967914395</v>
+        <v>564109.21054314391</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.25">
@@ -4576,11 +4574,11 @@
         <v>3.33</v>
       </c>
       <c r="G30" s="24">
-        <v>131782.53545009997</v>
+        <v>153258.16875300001</v>
       </c>
       <c r="H30" s="29">
         <f>G30</f>
-        <v>131782.53545009997</v>
+        <v>153258.16875300001</v>
       </c>
       <c r="I30" s="13" t="s">
         <v>123</v>
@@ -4595,16 +4593,16 @@
       </c>
       <c r="L30" s="6">
         <f t="shared" si="2"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="M30" s="23"/>
       <c r="N30" s="23">
         <f t="shared" si="4"/>
-        <v>153258.16875300001</v>
+        <v>248740.74360000002</v>
       </c>
       <c r="O30" s="23">
         <f t="shared" si="3"/>
-        <v>162453.65887817999</v>
+        <v>263665.18821600004</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.25">
@@ -4623,17 +4621,17 @@
         <v>3.24</v>
       </c>
       <c r="G31" s="24">
-        <v>762499.95606409316</v>
+        <v>783395.0121480932</v>
       </c>
       <c r="H31" s="29">
-        <v>128221</v>
+        <v>149116</v>
       </c>
       <c r="I31" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J31" s="7">
         <f t="shared" si="0"/>
-        <v>-634278.95606409316</v>
+        <v>-634279.0121480932</v>
       </c>
       <c r="K31" s="40">
         <f t="shared" si="1"/>
@@ -4641,16 +4639,16 @@
       </c>
       <c r="L31" s="6">
         <f t="shared" si="2"/>
-        <v>149116.05608400004</v>
+        <v>242018.02080000003</v>
       </c>
       <c r="M31" s="23"/>
       <c r="N31" s="23">
         <f>L31+K31-J31+M31</f>
-        <v>783395.0121480932</v>
+        <v>876297.03294809326</v>
       </c>
       <c r="O31" s="23">
         <f t="shared" si="3"/>
-        <v>830398.7128769788</v>
+        <v>928874.8549249788</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.25">
@@ -4669,11 +4667,11 @@
         <v>1.64</v>
       </c>
       <c r="G32" s="24">
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="H32" s="29">
         <f>G32</f>
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="I32" s="13" t="s">
         <v>123</v>
@@ -4688,16 +4686,16 @@
       </c>
       <c r="L32" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M32" s="23"/>
       <c r="N32" s="23">
         <f t="shared" si="4"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="O32" s="23">
         <f t="shared" si="3"/>
-        <v>80007.20737543999</v>
+        <v>129853.12572799998</v>
       </c>
     </row>
     <row r="33" spans="1:17" x14ac:dyDescent="0.25">
@@ -4716,11 +4714,11 @@
         <v>1.64</v>
       </c>
       <c r="G33" s="24">
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="H33" s="29">
         <f>G33</f>
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="I33" s="13" t="s">
         <v>123</v>
@@ -4735,16 +4733,16 @@
       </c>
       <c r="L33" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M33" s="23"/>
       <c r="N33" s="23">
         <f t="shared" si="4"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="O33" s="23">
         <f t="shared" si="3"/>
-        <v>80007.20737543999</v>
+        <v>129853.12572799998</v>
       </c>
     </row>
     <row r="34" spans="1:17" x14ac:dyDescent="0.25">
@@ -4763,17 +4761,17 @@
         <v>1.64</v>
       </c>
       <c r="G34" s="24">
-        <v>62185.339313367265</v>
+        <v>74663.836837367257</v>
       </c>
       <c r="H34" s="29">
-        <v>63000</v>
+        <v>65000</v>
       </c>
       <c r="I34" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J34" s="7">
         <f t="shared" si="0"/>
-        <v>814.66068663273472</v>
+        <v>-9663.8368373672565</v>
       </c>
       <c r="K34" s="40">
         <f t="shared" si="1"/>
@@ -4781,16 +4779,16 @@
       </c>
       <c r="L34" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M34" s="23"/>
       <c r="N34" s="23">
         <f t="shared" si="4"/>
-        <v>74663.836837367257</v>
+        <v>132166.78563736723</v>
       </c>
       <c r="O34" s="23">
         <f t="shared" si="3"/>
-        <v>79143.667047609284</v>
+        <v>140096.79277560927</v>
       </c>
     </row>
     <row r="35" spans="1:17" x14ac:dyDescent="0.25">
@@ -4809,7 +4807,7 @@
         <v>1.64</v>
       </c>
       <c r="G35" s="24">
-        <v>64901.909350799979</v>
+        <v>140380.40687479998</v>
       </c>
       <c r="H35" s="29"/>
       <c r="I35" s="13" t="s">
@@ -4817,7 +4815,7 @@
       </c>
       <c r="J35" s="7">
         <f t="shared" si="0"/>
-        <v>-64901.909350799979</v>
+        <v>-140380.40687479998</v>
       </c>
       <c r="K35" s="40">
         <f t="shared" si="1"/>
@@ -4825,19 +4823,19 @@
       </c>
       <c r="L35" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M35" s="23"/>
       <c r="N35" s="23">
         <f t="shared" si="4"/>
-        <v>140380.40687479998</v>
+        <v>262883.3556748</v>
       </c>
       <c r="O35" s="23">
         <f t="shared" si="3"/>
-        <v>148803.23128728798</v>
+        <v>278656.35701528797</v>
       </c>
       <c r="Q35" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.25">
@@ -4856,11 +4854,11 @@
         <v>1.64</v>
       </c>
       <c r="G36" s="24">
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="H36" s="29">
         <f>G36</f>
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="I36" s="13" t="s">
         <v>140</v>
@@ -4875,16 +4873,16 @@
       </c>
       <c r="L36" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M36" s="23"/>
       <c r="N36" s="23">
         <f t="shared" si="4"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="O36" s="23">
         <f t="shared" si="3"/>
-        <v>80007.20737543999</v>
+        <v>129853.12572799998</v>
       </c>
     </row>
     <row r="37" spans="1:17" x14ac:dyDescent="0.25">
@@ -4903,11 +4901,11 @@
         <v>1.64</v>
       </c>
       <c r="G37" s="24">
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="H37" s="29">
         <f>G37</f>
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="I37" s="13" t="s">
         <v>124</v>
@@ -4922,16 +4920,16 @@
       </c>
       <c r="L37" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M37" s="23"/>
       <c r="N37" s="23">
         <f t="shared" si="4"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="O37" s="23">
         <f t="shared" si="3"/>
-        <v>80007.20737543999</v>
+        <v>129853.12572799998</v>
       </c>
     </row>
     <row r="38" spans="1:17" x14ac:dyDescent="0.25">
@@ -4950,7 +4948,7 @@
         <v>1.64</v>
       </c>
       <c r="G38" s="24">
-        <v>917950.38750476763</v>
+        <v>993428.88502876763</v>
       </c>
       <c r="H38" s="29"/>
       <c r="I38" s="13" t="s">
@@ -4958,7 +4956,7 @@
       </c>
       <c r="J38" s="7">
         <f t="shared" si="0"/>
-        <v>-917950.38750476763</v>
+        <v>-993428.88502876763</v>
       </c>
       <c r="K38" s="40">
         <f t="shared" si="1"/>
@@ -4966,16 +4964,16 @@
       </c>
       <c r="L38" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M38" s="23"/>
       <c r="N38" s="23">
         <f t="shared" si="4"/>
-        <v>993428.88502876763</v>
+        <v>1115931.8338287675</v>
       </c>
       <c r="O38" s="23">
         <f t="shared" si="3"/>
-        <v>1053034.6181304937</v>
+        <v>1182887.7438584936</v>
       </c>
     </row>
     <row r="39" spans="1:17" x14ac:dyDescent="0.25">
@@ -4994,11 +4992,11 @@
         <v>1.64</v>
       </c>
       <c r="G39" s="24">
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="H39" s="29">
         <f>G39</f>
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="I39" s="13" t="s">
         <v>123</v>
@@ -5013,16 +5011,16 @@
       </c>
       <c r="L39" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M39" s="23"/>
       <c r="N39" s="23">
         <f t="shared" si="4"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="O39" s="23">
         <f t="shared" si="3"/>
-        <v>80007.20737543999</v>
+        <v>129853.12572799998</v>
       </c>
     </row>
     <row r="40" spans="1:17" x14ac:dyDescent="0.25">
@@ -5043,11 +5041,11 @@
         <v>1.64</v>
       </c>
       <c r="G40" s="24">
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="H40" s="29">
         <f>G40</f>
-        <v>64901.909350799979</v>
+        <v>75478.497523999991</v>
       </c>
       <c r="I40" s="13" t="s">
         <v>140</v>
@@ -5062,16 +5060,16 @@
       </c>
       <c r="L40" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M40" s="23"/>
       <c r="N40" s="23">
         <f t="shared" si="4"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="O40" s="23">
         <f t="shared" si="3"/>
-        <v>80007.20737543999</v>
+        <v>129853.12572799998</v>
       </c>
     </row>
     <row r="41" spans="1:17" x14ac:dyDescent="0.25">
@@ -5090,17 +5088,17 @@
         <v>1.64</v>
       </c>
       <c r="G41" s="24">
-        <v>61461.966481599899</v>
+        <v>71790.46400559989</v>
       </c>
       <c r="H41" s="29">
-        <v>65150</v>
+        <v>76098</v>
       </c>
       <c r="I41" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J41" s="7">
         <f t="shared" si="0"/>
-        <v>3688.0335184001015</v>
+        <v>4307.5359944001102</v>
       </c>
       <c r="K41" s="40">
         <f t="shared" si="1"/>
@@ -5108,16 +5106,16 @@
       </c>
       <c r="L41" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M41" s="23"/>
       <c r="N41" s="23">
         <f t="shared" si="4"/>
-        <v>71790.46400559989</v>
+        <v>118195.41280559987</v>
       </c>
       <c r="O41" s="23">
         <f t="shared" si="3"/>
-        <v>76097.891845935883</v>
+        <v>125287.13757393586</v>
       </c>
     </row>
     <row r="42" spans="1:17" x14ac:dyDescent="0.25">
@@ -5136,18 +5134,15 @@
         <v>1.64</v>
       </c>
       <c r="G42" s="24">
-        <v>194705.72805239994</v>
-      </c>
-      <c r="H42" s="29">
-        <f>131386</f>
-        <v>131386</v>
-      </c>
+        <v>138798.22557639994</v>
+      </c>
+      <c r="H42" s="29"/>
       <c r="I42" s="13" t="s">
         <v>123</v>
       </c>
       <c r="J42" s="7">
         <f t="shared" si="0"/>
-        <v>-63319.728052399936</v>
+        <v>-138798.22557639994</v>
       </c>
       <c r="K42" s="40">
         <f t="shared" si="1"/>
@@ -5155,16 +5150,16 @@
       </c>
       <c r="L42" s="6">
         <f t="shared" si="2"/>
-        <v>75478.497523999991</v>
+        <v>122502.94879999998</v>
       </c>
       <c r="M42" s="23"/>
       <c r="N42" s="23">
         <f t="shared" si="4"/>
-        <v>138798.22557639994</v>
+        <v>261301.17437639993</v>
       </c>
       <c r="O42" s="23">
         <f t="shared" si="3"/>
-        <v>147126.11911098394</v>
+        <v>276979.24483898393</v>
       </c>
     </row>
     <row r="43" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -5179,16 +5174,16 @@
       </c>
       <c r="G43" s="9">
         <f>SUM(G7:G42)</f>
-        <v>8389069.1426655836</v>
+        <v>9727292.9889031108</v>
       </c>
       <c r="H43" s="9">
         <f>SUM(H7:H42)</f>
-        <v>3277433.5524721928</v>
+        <v>3941990.5853970982</v>
       </c>
       <c r="I43" s="9"/>
       <c r="J43" s="139">
         <f t="shared" ref="J43:O43" si="5">SUM(J7:J42)</f>
-        <v>-5111635.5901933871</v>
+        <v>-5785302.403506008</v>
       </c>
       <c r="K43" s="9">
         <f t="shared" si="5"/>
@@ -5196,7 +5191,7 @@
       </c>
       <c r="L43" s="9">
         <f t="shared" si="5"/>
-        <v>4606489.5226689978</v>
+        <v>7476414.7228000024</v>
       </c>
       <c r="M43" s="8">
         <f t="shared" si="5"/>
@@ -5204,11 +5199,11 @@
       </c>
       <c r="N43" s="10">
         <f t="shared" si="5"/>
-        <v>9718125.1128623914</v>
+        <v>13261717.126306005</v>
       </c>
       <c r="O43" s="9">
         <f t="shared" si="5"/>
-        <v>10301212.619634137</v>
+        <v>14057420.15388437</v>
       </c>
     </row>
     <row r="44" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
@@ -5217,7 +5212,7 @@
       </c>
       <c r="I44">
         <f>SUMIF(I7:I42,"b",H7:H42)</f>
-        <v>2822724.5812739334</v>
+        <v>3413182.0317890993</v>
       </c>
       <c r="L44" s="11"/>
     </row>
@@ -5227,7 +5222,7 @@
       </c>
       <c r="I45">
         <f>SUMIF(I7:I42,"e",H7:H42)</f>
-        <v>454708.97119825997</v>
+        <v>528808.55360800005</v>
       </c>
     </row>
     <row r="46" spans="1:17" hidden="1" x14ac:dyDescent="0.25">
@@ -5236,91 +5231,97 @@
       </c>
       <c r="H46" s="36">
         <f>I44+I45</f>
-        <v>3277433.5524721933</v>
+        <v>3941990.5853970991</v>
       </c>
     </row>
     <row r="49" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D49" s="166" t="s">
+      <c r="D49" s="160" t="s">
         <v>182</v>
       </c>
-      <c r="E49" s="166"/>
-      <c r="F49" s="166"/>
-      <c r="G49" s="166"/>
-      <c r="H49" s="166"/>
-      <c r="I49" s="166"/>
-      <c r="J49" s="166"/>
-      <c r="K49" s="166"/>
-      <c r="L49" s="166"/>
-      <c r="M49" s="166"/>
-      <c r="N49" s="166"/>
+      <c r="E49" s="160"/>
+      <c r="F49" s="160"/>
+      <c r="G49" s="160"/>
+      <c r="H49" s="160"/>
+      <c r="I49" s="160"/>
+      <c r="J49" s="160"/>
+      <c r="K49" s="160"/>
+      <c r="L49" s="160"/>
+      <c r="M49" s="160"/>
+      <c r="N49" s="160"/>
     </row>
     <row r="50" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D50" s="166"/>
-      <c r="E50" s="166"/>
-      <c r="F50" s="166"/>
-      <c r="G50" s="166"/>
-      <c r="H50" s="166"/>
-      <c r="I50" s="166"/>
-      <c r="J50" s="166"/>
-      <c r="K50" s="166"/>
-      <c r="L50" s="166"/>
-      <c r="M50" s="166"/>
-      <c r="N50" s="166"/>
+      <c r="D50" s="160"/>
+      <c r="E50" s="160"/>
+      <c r="F50" s="160"/>
+      <c r="G50" s="160"/>
+      <c r="H50" s="160"/>
+      <c r="I50" s="160"/>
+      <c r="J50" s="160"/>
+      <c r="K50" s="160"/>
+      <c r="L50" s="160"/>
+      <c r="M50" s="160"/>
+      <c r="N50" s="160"/>
     </row>
     <row r="51" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D51" s="166"/>
-      <c r="E51" s="166"/>
-      <c r="F51" s="166"/>
-      <c r="G51" s="166"/>
-      <c r="H51" s="166"/>
-      <c r="I51" s="166"/>
-      <c r="J51" s="166"/>
-      <c r="K51" s="166"/>
-      <c r="L51" s="166"/>
-      <c r="M51" s="166"/>
-      <c r="N51" s="166"/>
+      <c r="D51" s="160"/>
+      <c r="E51" s="160"/>
+      <c r="F51" s="160"/>
+      <c r="G51" s="160"/>
+      <c r="H51" s="160"/>
+      <c r="I51" s="160"/>
+      <c r="J51" s="160"/>
+      <c r="K51" s="160"/>
+      <c r="L51" s="160"/>
+      <c r="M51" s="160"/>
+      <c r="N51" s="160"/>
     </row>
     <row r="52" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D52" s="166"/>
-      <c r="E52" s="166"/>
-      <c r="F52" s="166"/>
-      <c r="G52" s="166"/>
-      <c r="H52" s="166"/>
-      <c r="I52" s="166"/>
-      <c r="J52" s="166"/>
-      <c r="K52" s="166"/>
-      <c r="L52" s="166"/>
-      <c r="M52" s="166"/>
-      <c r="N52" s="166"/>
+      <c r="D52" s="160"/>
+      <c r="E52" s="160"/>
+      <c r="F52" s="160"/>
+      <c r="G52" s="160"/>
+      <c r="H52" s="160"/>
+      <c r="I52" s="160"/>
+      <c r="J52" s="160"/>
+      <c r="K52" s="160"/>
+      <c r="L52" s="160"/>
+      <c r="M52" s="160"/>
+      <c r="N52" s="160"/>
     </row>
     <row r="53" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D53" s="166"/>
-      <c r="E53" s="166"/>
-      <c r="F53" s="166"/>
-      <c r="G53" s="166"/>
-      <c r="H53" s="166"/>
-      <c r="I53" s="166"/>
-      <c r="J53" s="166"/>
-      <c r="K53" s="166"/>
-      <c r="L53" s="166"/>
-      <c r="M53" s="166"/>
-      <c r="N53" s="166"/>
+      <c r="D53" s="160"/>
+      <c r="E53" s="160"/>
+      <c r="F53" s="160"/>
+      <c r="G53" s="160"/>
+      <c r="H53" s="160"/>
+      <c r="I53" s="160"/>
+      <c r="J53" s="160"/>
+      <c r="K53" s="160"/>
+      <c r="L53" s="160"/>
+      <c r="M53" s="160"/>
+      <c r="N53" s="160"/>
     </row>
     <row r="54" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D54" s="166"/>
-      <c r="E54" s="166"/>
-      <c r="F54" s="166"/>
-      <c r="G54" s="166"/>
-      <c r="H54" s="166"/>
-      <c r="I54" s="166"/>
-      <c r="J54" s="166"/>
-      <c r="K54" s="166"/>
-      <c r="L54" s="166"/>
-      <c r="M54" s="166"/>
-      <c r="N54" s="166"/>
+      <c r="D54" s="160"/>
+      <c r="E54" s="160"/>
+      <c r="F54" s="160"/>
+      <c r="G54" s="160"/>
+      <c r="H54" s="160"/>
+      <c r="I54" s="160"/>
+      <c r="J54" s="160"/>
+      <c r="K54" s="160"/>
+      <c r="L54" s="160"/>
+      <c r="M54" s="160"/>
+      <c r="N54" s="160"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="D49:N54"/>
     <mergeCell ref="N4:O4"/>
     <mergeCell ref="N3:O3"/>
@@ -5332,12 +5333,6 @@
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="M5:M6"/>
     <mergeCell ref="N5:N6"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
@@ -5351,28 +5346,28 @@
   <sheetData>
     <row r="6" spans="5:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="7" spans="5:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E7" s="181" t="s">
+      <c r="E7" s="182" t="s">
         <v>165</v>
       </c>
-      <c r="F7" s="182"/>
-      <c r="G7" s="182"/>
-      <c r="H7" s="182"/>
-      <c r="I7" s="182"/>
-      <c r="J7" s="182"/>
-      <c r="K7" s="180"/>
+      <c r="F7" s="183"/>
+      <c r="G7" s="183"/>
+      <c r="H7" s="183"/>
+      <c r="I7" s="183"/>
+      <c r="J7" s="183"/>
+      <c r="K7" s="181"/>
       <c r="L7" s="44"/>
       <c r="M7" s="45"/>
     </row>
     <row r="8" spans="5:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E8" s="183" t="s">
+      <c r="E8" s="184" t="s">
         <v>166</v>
       </c>
-      <c r="F8" s="182"/>
-      <c r="G8" s="182"/>
-      <c r="H8" s="182"/>
-      <c r="I8" s="182"/>
-      <c r="J8" s="182"/>
-      <c r="K8" s="180"/>
+      <c r="F8" s="183"/>
+      <c r="G8" s="183"/>
+      <c r="H8" s="183"/>
+      <c r="I8" s="183"/>
+      <c r="J8" s="183"/>
+      <c r="K8" s="181"/>
       <c r="L8" s="46"/>
       <c r="M8" s="47"/>
     </row>
@@ -5416,15 +5411,15 @@
       <c r="M11" s="47"/>
     </row>
     <row r="12" spans="5:13" x14ac:dyDescent="0.25">
-      <c r="E12" s="184" t="s">
+      <c r="E12" s="185" t="s">
         <v>170</v>
       </c>
-      <c r="F12" s="185"/>
-      <c r="G12" s="185"/>
-      <c r="H12" s="185"/>
-      <c r="I12" s="185"/>
-      <c r="J12" s="185"/>
-      <c r="K12" s="186"/>
+      <c r="F12" s="186"/>
+      <c r="G12" s="186"/>
+      <c r="H12" s="186"/>
+      <c r="I12" s="186"/>
+      <c r="J12" s="186"/>
+      <c r="K12" s="187"/>
       <c r="L12" s="46"/>
       <c r="M12" s="47"/>
     </row>
@@ -5456,10 +5451,10 @@
         <v>45600</v>
       </c>
       <c r="K14" s="47"/>
-      <c r="L14" s="174" t="s">
+      <c r="L14" s="175" t="s">
         <v>173</v>
       </c>
-      <c r="M14" s="175"/>
+      <c r="M14" s="176"/>
     </row>
     <row r="15" spans="5:13" x14ac:dyDescent="0.25">
       <c r="E15" s="46" t="s">
@@ -5485,8 +5480,8 @@
       <c r="I16" s="49"/>
       <c r="J16" s="49"/>
       <c r="K16" s="47"/>
-      <c r="L16" s="176"/>
-      <c r="M16" s="175"/>
+      <c r="L16" s="177"/>
+      <c r="M16" s="176"/>
     </row>
     <row r="17" spans="5:15" x14ac:dyDescent="0.25">
       <c r="E17" s="46"/>
@@ -5522,45 +5517,45 @@
       <c r="M19" s="56"/>
     </row>
     <row r="20" spans="5:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="E20" s="177" t="s">
+      <c r="E20" s="178" t="s">
         <v>175</v>
       </c>
-      <c r="F20" s="178"/>
-      <c r="G20" s="178"/>
-      <c r="H20" s="178"/>
-      <c r="I20" s="178"/>
-      <c r="J20" s="179">
+      <c r="F20" s="179"/>
+      <c r="G20" s="179"/>
+      <c r="H20" s="179"/>
+      <c r="I20" s="179"/>
+      <c r="J20" s="180">
         <f>PRORRATEO!H12</f>
-        <v>131782.53545009997</v>
-      </c>
-      <c r="K20" s="180"/>
+        <v>153258.16875300001</v>
+      </c>
+      <c r="K20" s="181"/>
       <c r="L20" s="57"/>
       <c r="M20" s="58"/>
     </row>
     <row r="24" spans="5:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="25" spans="5:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G25" s="181" t="s">
+      <c r="G25" s="182" t="s">
         <v>165</v>
       </c>
-      <c r="H25" s="182"/>
-      <c r="I25" s="182"/>
-      <c r="J25" s="182"/>
-      <c r="K25" s="182"/>
-      <c r="L25" s="182"/>
-      <c r="M25" s="180"/>
+      <c r="H25" s="183"/>
+      <c r="I25" s="183"/>
+      <c r="J25" s="183"/>
+      <c r="K25" s="183"/>
+      <c r="L25" s="183"/>
+      <c r="M25" s="181"/>
       <c r="N25" s="44"/>
       <c r="O25" s="45"/>
     </row>
     <row r="26" spans="5:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G26" s="183" t="s">
+      <c r="G26" s="184" t="s">
         <v>166</v>
       </c>
-      <c r="H26" s="182"/>
-      <c r="I26" s="182"/>
-      <c r="J26" s="182"/>
-      <c r="K26" s="182"/>
-      <c r="L26" s="182"/>
-      <c r="M26" s="180"/>
+      <c r="H26" s="183"/>
+      <c r="I26" s="183"/>
+      <c r="J26" s="183"/>
+      <c r="K26" s="183"/>
+      <c r="L26" s="183"/>
+      <c r="M26" s="181"/>
       <c r="N26" s="46"/>
       <c r="O26" s="47"/>
     </row>
@@ -5604,15 +5599,15 @@
       <c r="O29" s="47"/>
     </row>
     <row r="30" spans="5:15" x14ac:dyDescent="0.25">
-      <c r="G30" s="184" t="s">
+      <c r="G30" s="185" t="s">
         <v>170</v>
       </c>
-      <c r="H30" s="185"/>
-      <c r="I30" s="185"/>
-      <c r="J30" s="185"/>
-      <c r="K30" s="185"/>
-      <c r="L30" s="185"/>
-      <c r="M30" s="186"/>
+      <c r="H30" s="186"/>
+      <c r="I30" s="186"/>
+      <c r="J30" s="186"/>
+      <c r="K30" s="186"/>
+      <c r="L30" s="186"/>
+      <c r="M30" s="187"/>
       <c r="N30" s="46"/>
       <c r="O30" s="47"/>
     </row>
@@ -5641,10 +5636,10 @@
         <v>45600</v>
       </c>
       <c r="M32" s="47"/>
-      <c r="N32" s="174" t="s">
+      <c r="N32" s="175" t="s">
         <v>173</v>
       </c>
-      <c r="O32" s="175"/>
+      <c r="O32" s="176"/>
     </row>
     <row r="33" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G33" s="46" t="s">
@@ -5670,8 +5665,8 @@
       <c r="K34" s="49"/>
       <c r="L34" s="49"/>
       <c r="M34" s="47"/>
-      <c r="N34" s="176"/>
-      <c r="O34" s="175"/>
+      <c r="N34" s="177"/>
+      <c r="O34" s="176"/>
     </row>
     <row r="35" spans="7:15" x14ac:dyDescent="0.25">
       <c r="G35" s="46"/>
@@ -5707,18 +5702,18 @@
       <c r="O37" s="56"/>
     </row>
     <row r="38" spans="7:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G38" s="177" t="s">
+      <c r="G38" s="178" t="s">
         <v>175</v>
       </c>
-      <c r="H38" s="178"/>
-      <c r="I38" s="178"/>
-      <c r="J38" s="178"/>
-      <c r="K38" s="178"/>
-      <c r="L38" s="179">
+      <c r="H38" s="179"/>
+      <c r="I38" s="179"/>
+      <c r="J38" s="179"/>
+      <c r="K38" s="179"/>
+      <c r="L38" s="180">
         <f>PRORRATEO!J30</f>
         <v>0</v>
       </c>
-      <c r="M38" s="180"/>
+      <c r="M38" s="181"/>
       <c r="N38" s="57"/>
       <c r="O38" s="58"/>
     </row>

</xml_diff>